<commit_message>
Update App Content via Excel
</commit_message>
<xml_diff>
--- a/Update_App_Data/upsc_toppers_data.xlsx
+++ b/Update_App_Data/upsc_toppers_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFC51479-CD82-4AFA-9521-A6378C7AE4A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9095A555-BDD8-468E-B121-9581D4812911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Strategy" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="106">
   <si>
     <t>id</t>
   </si>
@@ -88,54 +88,9 @@
     <t>goldenRules</t>
   </si>
   <si>
-    <t>aditya-srivastava</t>
-  </si>
-  <si>
     <t>Aditya Srivastava</t>
   </si>
   <si>
-    <t>Electrical Engineering</t>
-  </si>
-  <si>
-    <t>B.Tech IIT Kanpur (Ex-Goldman Sachs &amp; Ex-IPS)</t>
-  </si>
-  <si>
-    <t>https://images.unsplash.com/photo-1534528741775-53994a69daeb?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
-  </si>
-  <si>
-    <t>Mains is all about smart presentation, precise micro-diagrams, and time management. Every half mark accumulated across 20 questions makes the difference between AIR 1 and missing the list.</t>
-  </si>
-  <si>
-    <t>Treated UPSC preparation as a structured engineering optimization problem. Focused heavily on PYQ reverse-engineering, creating concise 1-page notes for every syllabus keyword, and rigorous timed full-length test simulations.</t>
-  </si>
-  <si>
-    <t>History through timelines and maps; Geography with crisp schematic drawings; Society with recent Census data, NFHS-5 surveys, and committee reports.</t>
-  </si>
-  <si>
-    <t>Directly mapped every constitutional article, Supreme Court 2nd &amp; 3rd ARC recommendations, and punchy international relations 2x2 matrices.</t>
-  </si>
-  <si>
-    <t>Focus on Economic Survey graphs, NITI Aayog Strategy for New India metrics, science &amp; tech contemporary applications, and internal security maps.</t>
-  </si>
-  <si>
-    <t>Prepared a personal repository of 50 real-life civil servant examples, philosophical quotes with applied meanings, and standard 7-step case study stakeholder resolution framework.</t>
-  </si>
-  <si>
-    <t>Wrote multi-dimensional essays exploring Historical, Social, Economic, Political, Psychological, and Ethical angles (PESTLE + philosophical lens). Used catchy quotes in intro and closed with inspirational vision.</t>
-  </si>
-  <si>
-    <t>Mastered electrical engineering fundamentals through rigorous numerical problem-solving and clean circuit diagrams. Practiced 10 years PYQs thrice.</t>
-  </si>
-  <si>
-    <t>Solved 60+ full length mock tests. Analyzed every incorrect option thoroughly. Maintained 90+ attempts with a calculated intelligent elimination approach.</t>
-  </si>
-  <si>
-    <t>Practiced 30 minutes daily from January onwards. Prioritized high-accuracy reading comprehension and quant problem patterns.</t>
-  </si>
-  <si>
-    <t>Limit your resources: 1 book read 10 times is better than 10 books read once. | Never write an answer without at least 1 diagram/flowchart or data point. | Syllabus keywords are your holy grail: prepare 150-word notes for each keyword. | Consistency over intensity: 7 focused hours daily beats erratic 14-hour burnout.</t>
-  </si>
-  <si>
     <t>ishita-kishore</t>
   </si>
   <si>
@@ -148,9 +103,6 @@
     <t>BA (Hons) Economics, SRCC Delhi (National Football Player)</t>
   </si>
   <si>
-    <t>https://images.unsplash.com/photo-1573496359142-b8d87734a5a2?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
-  </si>
-  <si>
     <t>Failures are simply data points showing where to refine your technique. After two prelims failures, fixing my active recall and mock test feedback loop changed everything.</t>
   </si>
   <si>
@@ -232,102 +184,6 @@
     <t>Consolidate your own notes for every single line of the syllabus. | PYQs are the best teacher: study the options that UPSC eliminated in previous years. | Write answer copies in the actual UPSC format with margins. | Keep answers balanced, objective, and constructive.</t>
   </si>
   <si>
-    <t>shubham-kumar</t>
-  </si>
-  <si>
-    <t>Shubham Kumar</t>
-  </si>
-  <si>
-    <t>Anthropology</t>
-  </si>
-  <si>
-    <t>B.Tech IIT Bombay (Civil Engineering)</t>
-  </si>
-  <si>
-    <t>https://images.unsplash.com/photo-1507003211169-0a1dd7228f2d?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
-  </si>
-  <si>
-    <t>Stick to the basics and optimize your optional. Anthropology diagrams and case studies gave me the decisive scoring edge.</t>
-  </si>
-  <si>
-    <t>High scoring in Optional (320+) and GS3/GS4. Mastered fast diagramming techniques in Mains, completing every single paper on time.</t>
-  </si>
-  <si>
-    <t>Brief intro + 2 neat subheadings + map/diagram + 1 line balanced conclusion.</t>
-  </si>
-  <si>
-    <t>Articles highlighted with boxes, ARC-2 recommendations, NITI Aayog indices.</t>
-  </si>
-  <si>
-    <t>High-scoring graphs for inflation, GDP trends, and agriculture marketing.</t>
-  </si>
-  <si>
-    <t>Practical ethical analysis with clear stakeholder matrices.</t>
-  </si>
-  <si>
-    <t>Structured essays with catchy thematic titles, real stories from rural India, and concrete policy recommendations.</t>
-  </si>
-  <si>
-    <t>Prepared over 150 biological and socio-cultural anthropology diagrams that could be drawn in under 45 seconds.</t>
-  </si>
-  <si>
-    <t>Practiced 75+ mocks. Focused heavily on high-weightage pillars (Polity, Modern History, Economy, Environment).</t>
-  </si>
-  <si>
-    <t>Strong focus on quant speed techniques and data interpretation.</t>
-  </si>
-  <si>
-    <t>Draw diagrams in at least 12 out of 20 questions in every GS paper. | Time management is supreme: 7 mins for 10-markers, 11 mins for 15-markers. | Revise high-weightage static subjects before touching new current affairs. | Maintain physical discipline through daily running and meditation.</t>
-  </si>
-  <si>
-    <t>kanishak-kataria</t>
-  </si>
-  <si>
-    <t>Kanishak Kataria</t>
-  </si>
-  <si>
-    <t>Mathematics</t>
-  </si>
-  <si>
-    <t>B.Tech IIT Bombay (Computer Science &amp; Engineering)</t>
-  </si>
-  <si>
-    <t>https://images.unsplash.com/photo-1500648767791-00dcc994a43e?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
-  </si>
-  <si>
-    <t>Objectivity is the key to UPSC Mains. Write what is asked, not what you know. Keep sentences short, data-backed, and use flowcharts whenever possible to save time.</t>
-  </si>
-  <si>
-    <t>Scored massively in Mathematics Optional (361/500). Prepared digitally using Evernote and OneNote, categorizing notes strictly by the UPSC syllabus keywords. Focused completely on high return on investment subjects like Ethics, Essay, and Optional.</t>
-  </si>
-  <si>
-    <t>Relied entirely on standard books. For Geography, practiced rapid map drawing for every location-based concept.</t>
-  </si>
-  <si>
-    <t>Used sub-headings aggressively. Quoted specific Articles, Constitutional Amendments, and Supreme Court judgements in every answer.</t>
-  </si>
-  <si>
-    <t>Treated GS3 like a technical paper. Filled answers with facts, figures, NITI Aayog data points, and block diagrams.</t>
-  </si>
-  <si>
-    <t>Prepared a personal list of core values and associated them with real-life administrative examples. Kept case studies structured and purely logical.</t>
-  </si>
-  <si>
-    <t>Brainstormed for 25 minutes before starting. Focused on logical flow, transitions between paragraphs, and maintaining a balanced, optimistic tone throughout.</t>
-  </si>
-  <si>
-    <t>Mathematics demands absolute rigor. Solved 15-20 years of PYQs. Made formula sheets for quick revision and practiced under strict time constraints to avoid calculation errors.</t>
-  </si>
-  <si>
-    <t>Did not over-read. Limited sources but revised them 5-6 times. Solved around 50 mock tests to develop the intuition for intelligent guessing and elimination.</t>
-  </si>
-  <si>
-    <t>Being from a math background, relied on natural aptitude but still practiced a few PYQs to stay in touch with the UPSC question phrasing.</t>
-  </si>
-  <si>
-    <t>Digital notes are easier to update, organize, and revise quickly. | Mathematics optional requires solving problems with pen and paper, not just reading solutions. | Focus intensely on your Optional, Essay, and Ethics—these create the rank difference. | Do not try to read everything; stick to the syllabus boundaries strictly.</t>
-  </si>
-  <si>
     <t>routineId</t>
   </si>
   <si>
@@ -482,6 +338,9 @@
   </si>
   <si>
     <t>DAF / Work Experience</t>
+  </si>
+  <si>
+    <t>https://www.google.com/imgres?q=avatar%20of%20ias&amp;imgurl=https%3A%2F%2Fpbs.twimg.com%2Fprofile_images%2F1261234351527866369%2FAMfcadQ8_400x400.jpg&amp;imgrefurl=https%3A%2F%2Fx.com%2Fiaskumaranurag&amp;docid=wjTnur9UPhOlyM&amp;tbnid=1PxNXllBXjuf2M&amp;vet=12ahUKEwj3uLPLo-aWAxVET2wGHe9eJA8QnPAOegQIQhAA..i&amp;w=400&amp;h=400&amp;hcb=2&amp;ved=2ahUKEwj3uLPLo-aWAxVET2wGHe9eJA8QnPAOegQIQhAA</t>
   </si>
 </sst>
 </file>
@@ -517,10 +376,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -861,403 +726,218 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:U3"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="11" style="3"/>
+    <col min="3" max="6" width="11" style="2"/>
+    <col min="7" max="7" width="11" style="3"/>
+    <col min="8" max="8" width="46.375" style="3" customWidth="1"/>
+    <col min="9" max="18" width="19.5" style="3" customWidth="1"/>
+    <col min="19" max="20" width="11" style="3"/>
+    <col min="21" max="21" width="40.625" style="3" customWidth="1"/>
+    <col min="22" max="16384" width="11" style="2"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:21" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="2" spans="1:21" ht="220.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C2">
+      <c r="B2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="2">
         <v>1</v>
       </c>
-      <c r="D2">
-        <v>2023</v>
-      </c>
-      <c r="E2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2">
+      <c r="D2" s="2">
+        <v>2022</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="2">
         <v>3</v>
       </c>
-      <c r="G2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="G2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H2" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="S2">
-        <v>200</v>
-      </c>
-      <c r="T2">
-        <v>899</v>
-      </c>
-      <c r="U2" t="s">
+      <c r="S2" s="3">
+        <v>193</v>
+      </c>
+      <c r="T2" s="3">
+        <v>901</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:21" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>2022</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="D3" s="2">
+        <v>2021</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="F3" s="2">
+        <v>2</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="S3">
-        <v>193</v>
-      </c>
-      <c r="T3">
-        <v>901</v>
-      </c>
-      <c r="U3" t="s">
+      <c r="S3" s="3">
+        <v>173</v>
+      </c>
+      <c r="T3" s="3">
+        <v>932</v>
+      </c>
+      <c r="U3" s="3" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>2021</v>
-      </c>
-      <c r="E4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="G4" t="s">
-        <v>56</v>
-      </c>
-      <c r="H4" t="s">
-        <v>57</v>
-      </c>
-      <c r="I4" t="s">
-        <v>58</v>
-      </c>
-      <c r="J4" t="s">
-        <v>59</v>
-      </c>
-      <c r="K4" t="s">
-        <v>60</v>
-      </c>
-      <c r="L4" t="s">
-        <v>61</v>
-      </c>
-      <c r="M4" t="s">
-        <v>62</v>
-      </c>
-      <c r="N4" t="s">
-        <v>63</v>
-      </c>
-      <c r="O4" t="s">
-        <v>64</v>
-      </c>
-      <c r="P4" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>66</v>
-      </c>
-      <c r="R4" t="s">
-        <v>67</v>
-      </c>
-      <c r="S4">
-        <v>173</v>
-      </c>
-      <c r="T4">
-        <v>932</v>
-      </c>
-      <c r="U4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>2020</v>
-      </c>
-      <c r="E5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5" t="s">
-        <v>72</v>
-      </c>
-      <c r="H5" t="s">
-        <v>73</v>
-      </c>
-      <c r="I5" t="s">
-        <v>74</v>
-      </c>
-      <c r="J5" t="s">
-        <v>75</v>
-      </c>
-      <c r="K5" t="s">
-        <v>76</v>
-      </c>
-      <c r="L5" t="s">
-        <v>77</v>
-      </c>
-      <c r="M5" t="s">
-        <v>78</v>
-      </c>
-      <c r="N5" t="s">
-        <v>79</v>
-      </c>
-      <c r="O5" t="s">
-        <v>80</v>
-      </c>
-      <c r="P5" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>82</v>
-      </c>
-      <c r="R5" t="s">
-        <v>83</v>
-      </c>
-      <c r="S5">
-        <v>176</v>
-      </c>
-      <c r="T5">
-        <v>878</v>
-      </c>
-      <c r="U5" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>2018</v>
-      </c>
-      <c r="E6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
-        <v>88</v>
-      </c>
-      <c r="H6" t="s">
-        <v>89</v>
-      </c>
-      <c r="I6" t="s">
-        <v>90</v>
-      </c>
-      <c r="J6" t="s">
-        <v>91</v>
-      </c>
-      <c r="K6" t="s">
-        <v>92</v>
-      </c>
-      <c r="L6" t="s">
-        <v>93</v>
-      </c>
-      <c r="M6" t="s">
-        <v>94</v>
-      </c>
-      <c r="N6" t="s">
-        <v>95</v>
-      </c>
-      <c r="O6" t="s">
-        <v>96</v>
-      </c>
-      <c r="P6" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>98</v>
-      </c>
-      <c r="R6" t="s">
-        <v>99</v>
-      </c>
-      <c r="S6">
-        <v>179</v>
-      </c>
-      <c r="T6">
-        <v>942</v>
-      </c>
-      <c r="U6" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:U6" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:U1 A3:U3 A2:G2 I2:U2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1265,7 +945,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1276,226 +956,225 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>101</v>
+        <v>53</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>103</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
-        <v>105</v>
+        <v>57</v>
       </c>
       <c r="F1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>115</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
       <c r="D3" t="s">
-        <v>116</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s">
-        <v>117</v>
+        <v>69</v>
       </c>
       <c r="F3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>119</v>
+        <v>71</v>
       </c>
       <c r="F4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
       <c r="D5" t="s">
-        <v>120</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
-        <v>121</v>
+        <v>73</v>
       </c>
       <c r="F5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
       <c r="D6" t="s">
-        <v>122</v>
+        <v>74</v>
       </c>
       <c r="E6" t="s">
-        <v>123</v>
+        <v>75</v>
       </c>
       <c r="F6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>76</v>
       </c>
       <c r="E7" t="s">
-        <v>125</v>
+        <v>77</v>
       </c>
       <c r="F7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>78</v>
       </c>
       <c r="E8" t="s">
-        <v>127</v>
+        <v>79</v>
       </c>
       <c r="F8" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>128</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>129</v>
+        <v>81</v>
       </c>
       <c r="E9" t="s">
-        <v>130</v>
+        <v>82</v>
       </c>
       <c r="F9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>128</v>
+        <v>80</v>
       </c>
       <c r="D10" t="s">
-        <v>131</v>
+        <v>83</v>
       </c>
       <c r="E10" t="s">
-        <v>132</v>
+        <v>84</v>
       </c>
       <c r="F10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>128</v>
+        <v>80</v>
       </c>
       <c r="D11" t="s">
-        <v>110</v>
+        <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>133</v>
+        <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>128</v>
+        <v>80</v>
       </c>
       <c r="D12" t="s">
-        <v>134</v>
+        <v>86</v>
       </c>
       <c r="E12" t="s">
-        <v>135</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>128</v>
+        <v>80</v>
       </c>
       <c r="D13" t="s">
-        <v>136</v>
+        <v>88</v>
       </c>
       <c r="E13" t="s">
-        <v>137</v>
+        <v>89</v>
       </c>
       <c r="F13" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>128</v>
+        <v>80</v>
       </c>
       <c r="D14" t="s">
-        <v>138</v>
+        <v>90</v>
       </c>
       <c r="E14" t="s">
-        <v>139</v>
+        <v>91</v>
       </c>
       <c r="F14" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>128</v>
+        <v>80</v>
       </c>
       <c r="D15" t="s">
-        <v>140</v>
+        <v>92</v>
       </c>
       <c r="E15" t="s">
-        <v>141</v>
+        <v>93</v>
       </c>
       <c r="F15" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25"/>
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1523,36 +1202,36 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>142</v>
+        <v>94</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>143</v>
+        <v>95</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>144</v>
+        <v>96</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>145</v>
+        <v>97</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>146</v>
+        <v>98</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>147</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>148</v>
+        <v>100</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>149</v>
+        <v>101</v>
       </c>
       <c r="D2" s="1">
         <v>2023</v>
@@ -1561,13 +1240,13 @@
         <v>200</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>150</v>
+        <v>102</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>151</v>
+        <v>103</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>152</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>